<commit_message>
worked on BCM ECU, removed 12V regs since not needed
</commit_message>
<xml_diff>
--- a/1_BCM_ECU/3_BCM_ECU_revA/BCM_ECU_CHANNEL_PINOUT.xlsx
+++ b/1_BCM_ECU/3_BCM_ECU_revA/BCM_ECU_CHANNEL_PINOUT.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\se097192\Documents\0_BRZ\BRZ_HARDWARE\1_BCM_ECU\3_BCM_ECU_revA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Trololololol\Documents\Projects\0_BRZ_PARENT\1_BRZ_HARDWARE\1_BCM_ECU\3_BCM_ECU_revA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BB0DDC1-6A0E-4B68-961C-80199A3BE4B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86258722-66C9-49FB-BD0F-D9E0347DB324}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="2415" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PWR CHANNELS" sheetId="1" r:id="rId1"/>
     <sheet name="LED CHANNELS" sheetId="2" r:id="rId2"/>
+    <sheet name="CONNECTOR PINOUTS" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="34">
   <si>
     <t>FUNCTION</t>
   </si>
@@ -130,6 +131,15 @@
   </si>
   <si>
     <t>?</t>
+  </si>
+  <si>
+    <t>CONN A</t>
+  </si>
+  <si>
+    <t>PIN #</t>
+  </si>
+  <si>
+    <t>PWR IN</t>
   </si>
 </sst>
 </file>
@@ -145,12 +155,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -165,8 +187,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -794,4 +821,237 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C24C731B-0870-43DB-9526-4D708776A2B5}">
+  <dimension ref="A1:N8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="1"/>
+      <c r="B1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="1"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="3">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <v>6</v>
+      </c>
+      <c r="H2">
+        <v>7</v>
+      </c>
+      <c r="I2">
+        <v>8</v>
+      </c>
+      <c r="J2">
+        <f>I2+1</f>
+        <v>9</v>
+      </c>
+      <c r="K2">
+        <f t="shared" ref="K2:M2" si="0">J2+1</f>
+        <v>10</v>
+      </c>
+      <c r="L2">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="M2">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="N2" s="1"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="N3" s="1"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="3">
+        <v>13</v>
+      </c>
+      <c r="C4" s="3">
+        <f>B4+1</f>
+        <v>14</v>
+      </c>
+      <c r="D4">
+        <f t="shared" ref="D4:L4" si="1">C4+1</f>
+        <v>15</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="1"/>
+        <v>16</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="1"/>
+        <v>17</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="1"/>
+        <v>18</v>
+      </c>
+      <c r="H4">
+        <f t="shared" si="1"/>
+        <v>19</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="1"/>
+        <v>21</v>
+      </c>
+      <c r="K4">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+      <c r="L4">
+        <f t="shared" si="1"/>
+        <v>23</v>
+      </c>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="3">
+        <v>24</v>
+      </c>
+      <c r="C6" s="3">
+        <f>B6+1</f>
+        <v>25</v>
+      </c>
+      <c r="D6">
+        <f t="shared" ref="D6:M6" si="2">C6+1</f>
+        <v>26</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="2"/>
+        <v>27</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="2"/>
+        <v>28</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="2"/>
+        <v>29</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="2"/>
+        <v>31</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="2"/>
+        <v>32</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="2"/>
+        <v>33</v>
+      </c>
+      <c r="L6">
+        <f t="shared" si="2"/>
+        <v>34</v>
+      </c>
+      <c r="M6">
+        <f t="shared" si="2"/>
+        <v>35</v>
+      </c>
+      <c r="N6" s="1"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="N7" s="1"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:M1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>